<commit_message>
Restaura apresentação do exemplo com alturas ajustadas e sem painéis congelados
</commit_message>
<xml_diff>
--- a/na-pratica/conciliacao-financeira/demonstrativo-exemplo.xlsx
+++ b/na-pratica/conciliacao-financeira/demonstrativo-exemplo.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exemplo fictício" sheetId="1" r:id="R18d72e02e2e2495f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exemplo fictício" sheetId="1" r:id="Rd7fe56b748174f15"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,29 +14,23 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:numFmts count="2">
-    <x:numFmt numFmtId="200" formatCode="dd/mm/yyyy"/>
-    <x:numFmt numFmtId="201" formatCode="&quot;R$ &quot;#,##0.00;[Red]&quot;-R$ &quot;#,##0.00"/>
+    <x:numFmt numFmtId="200" formatCode="&quot;R$ &quot;#,##0.00;[Red]&quot;-R$ &quot;#,##0.00"/>
+    <x:numFmt numFmtId="201" formatCode="dd/mm/yyyy"/>
   </x:numFmts>
-  <x:fonts count="10">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
+      <x:color rgb="FF17365D"/>
       <x:name val="Calibri"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="16"/>
       <x:color rgb="FFFFFFFF"/>
-      <x:name val="Calibri"/>
-    </x:font>
-    <x:font>
-      <x:i/>
-      <x:sz val="10"/>
-      <x:color rgb="FF666666"/>
       <x:name val="Calibri"/>
     </x:font>
     <x:font>
@@ -48,13 +42,7 @@
     <x:font>
       <x:b/>
       <x:sz val="11"/>
-      <x:color rgb="FF006100"/>
-      <x:name val="Calibri"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="10"/>
-      <x:color rgb="FF666666"/>
+      <x:color rgb="FF9C6500"/>
       <x:name val="Calibri"/>
     </x:font>
     <x:font>
@@ -63,19 +51,8 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Calibri"/>
     </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-    </x:font>
-    <x:font>
-      <x:sz val="10"/>
-      <x:color rgb="FF595959"/>
-      <x:name val="Calibri"/>
-    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -94,12 +71,7 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFFF00"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFE2F0D9"/>
+        <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -134,7 +106,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="43">
+  <x:cellXfs count="41">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -149,115 +121,109 @@
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="200" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="200" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -462,190 +428,202 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="68" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="52" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="19" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="54" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="38" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="21" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="52" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="36" customHeight="1">
+    <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>DEMONSTRATIVO FINANCEIRO - SETEMBRO 2026 - EXEMPLO FICTÍCIO</x:v>
+        <x:v>DEMONSTRATIVO FINANCEIRO - EXEMPLO INTEIRAMENTE FICTÍCIO</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
       <x:c r="D1" s="5"/>
       <x:c r="E1" s="5"/>
       <x:c r="F1" s="5"/>
-    </x:row>
-    <x:row r="2" ht="24" customHeight="1">
-      <x:c r="A2" s="6" t="str">
-        <x:v>Dados inteiramente fictícios: valores, partes, conta e documentos criados para demonstração.</x:v>
-      </x:c>
-      <x:c r="B2" s="6"/>
-      <x:c r="C2" s="6"/>
-      <x:c r="D2" s="6"/>
-      <x:c r="E2" s="6"/>
-      <x:c r="F2" s="6"/>
-    </x:row>
-    <x:row r="3" ht="25" customHeight="1">
-      <x:c r="A3" s="11" t="str">
+      <x:c r="G1" s="5"/>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="2" t="str">
+        <x:v>Ilustração pública. Valores, partes e documentos inventados para demonstração.</x:v>
+      </x:c>
+      <x:c r="B2" s="2"/>
+      <x:c r="C2" s="2"/>
+      <x:c r="D2" s="2"/>
+      <x:c r="E2" s="2"/>
+      <x:c r="F2" s="2"/>
+      <x:c r="G2" s="2"/>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="2"/>
+      <x:c r="B3" s="2"/>
+      <x:c r="C3" s="2"/>
+      <x:c r="D3" s="2"/>
+      <x:c r="E3" s="2"/>
+      <x:c r="F3" s="2"/>
+      <x:c r="G3" s="2"/>
+    </x:row>
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A4" s="8" t="str">
+        <x:v>Empresa</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="str">
+        <x:v>Empresa de demonstração</x:v>
+      </x:c>
+      <x:c r="C4" s="2"/>
+      <x:c r="D4" s="8" t="str">
+        <x:v>Saldo inicial</x:v>
+      </x:c>
+      <x:c r="E4" s="11" t="n">
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="F4" s="12" t="str">
+        <x:v>Base do exemplo</x:v>
+      </x:c>
+      <x:c r="G4" s="13" t="n">
+        <x:f>ROUND(SUM(F13:F24),2)</x:f>
+        <x:v>7500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="8" t="str">
         <x:v>Moeda</x:v>
       </x:c>
-      <x:c r="B3" s="8" t="str">
+      <x:c r="B5" s="2" t="str">
         <x:v>BRL</x:v>
       </x:c>
-      <x:c r="C3" s="2"/>
-      <x:c r="D3" s="11" t="str">
-        <x:v>Saldo inicial</x:v>
-      </x:c>
-      <x:c r="E3" s="12" t="n">
-        <x:v>12000</x:v>
-      </x:c>
-      <x:c r="F3" s="2"/>
-    </x:row>
-    <x:row r="4" ht="25" customHeight="1">
-      <x:c r="A4" s="11" t="str">
-        <x:v>Código bancário</x:v>
-      </x:c>
-      <x:c r="B4" s="8" t="str">
-        <x:v>Fictício</x:v>
-      </x:c>
-      <x:c r="C4" s="2"/>
-      <x:c r="D4" s="11" t="str">
-        <x:v>Total entradas</x:v>
-      </x:c>
-      <x:c r="E4" s="12" t="n">
+      <x:c r="C5" s="2"/>
+      <x:c r="D5" s="8" t="str">
+        <x:v>Entradas</x:v>
+      </x:c>
+      <x:c r="E5" s="11" t="n">
         <x:f>ROUND(SUMIF(A13:A24,"CREDIT",C13:C24),2)</x:f>
         <x:v>15000</x:v>
       </x:c>
-      <x:c r="F4" s="2"/>
-    </x:row>
-    <x:row r="5" ht="25" customHeight="1">
-      <x:c r="A5" s="11" t="str">
-        <x:v>Nome do banco</x:v>
-      </x:c>
-      <x:c r="B5" s="8" t="str">
-        <x:v>Banco de demonstração</x:v>
-      </x:c>
-      <x:c r="C5" s="2"/>
-      <x:c r="D5" s="11" t="str">
-        <x:v>Total saídas</x:v>
-      </x:c>
-      <x:c r="E5" s="12" t="n">
+      <x:c r="F5" s="8" t="str">
+        <x:v>Conciliação</x:v>
+      </x:c>
+      <x:c r="G5" s="2" t="str">
+        <x:f>IF(ABS(E9)&lt;=0.01,"OK","DIVERGENTE")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="8" t="str">
+        <x:v>Período</x:v>
+      </x:c>
+      <x:c r="B6" s="2" t="str">
+        <x:v>Setembro/2026</x:v>
+      </x:c>
+      <x:c r="C6" s="2"/>
+      <x:c r="D6" s="8" t="str">
+        <x:v>Saídas</x:v>
+      </x:c>
+      <x:c r="E6" s="11" t="n">
         <x:f>ROUND(-SUMIF(A13:A24,"PAYMENT",C13:C24),2)</x:f>
         <x:v>7320</x:v>
       </x:c>
-      <x:c r="F5" s="2"/>
-    </x:row>
-    <x:row r="6" ht="25" customHeight="1">
-      <x:c r="A6" s="11" t="str">
-        <x:v>Conta</x:v>
-      </x:c>
-      <x:c r="B6" s="8" t="str">
-        <x:v>CONTA FICTÍCIA</x:v>
-      </x:c>
-      <x:c r="C6" s="2"/>
-      <x:c r="D6" s="11" t="str">
+      <x:c r="F6" s="2"/>
+      <x:c r="G6" s="2"/>
+    </x:row>
+    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A7" s="8" t="str">
+        <x:v>Movimentos bancários</x:v>
+      </x:c>
+      <x:c r="B7" s="2" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C7" s="2"/>
+      <x:c r="D7" s="8" t="str">
         <x:v>Saldo final calculado</x:v>
       </x:c>
-      <x:c r="E6" s="12" t="n">
-        <x:f>ROUND(E3+E4-E5,2)</x:f>
+      <x:c r="E7" s="11" t="n">
+        <x:f>ROUND(E4+E5-E6,2)</x:f>
         <x:v>19680</x:v>
       </x:c>
-      <x:c r="F6" s="2"/>
-    </x:row>
-    <x:row r="7" ht="25" customHeight="1">
-      <x:c r="A7" s="11" t="str">
-        <x:v>Data inicial</x:v>
-      </x:c>
-      <x:c r="B7" s="9" t="d">
-        <x:v>2026-09-01T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C7" s="2"/>
-      <x:c r="D7" s="13" t="str">
-        <x:v>Base do exemplo</x:v>
-      </x:c>
-      <x:c r="E7" s="14" t="n">
-        <x:f>ROUND(SUM(F13:F24),2)</x:f>
-        <x:v>7500</x:v>
-      </x:c>
       <x:c r="F7" s="2"/>
-    </x:row>
-    <x:row r="8" ht="25" customHeight="1">
-      <x:c r="A8" s="11" t="str">
-        <x:v>Data final</x:v>
-      </x:c>
-      <x:c r="B8" s="9" t="d">
-        <x:v>2026-09-30T00:00:00.000Z</x:v>
+      <x:c r="G7" s="2"/>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="8" t="str">
+        <x:v>Linhas de detalhe</x:v>
+      </x:c>
+      <x:c r="B8" s="2" t="n">
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C8" s="2"/>
-      <x:c r="D8" s="11" t="str">
+      <x:c r="D8" s="8" t="str">
         <x:v>Saldo final de referência</x:v>
       </x:c>
-      <x:c r="E8" s="12" t="n">
+      <x:c r="E8" s="11" t="n">
         <x:v>19680</x:v>
       </x:c>
       <x:c r="F8" s="2"/>
-    </x:row>
-    <x:row r="9" ht="25" customHeight="1">
-      <x:c r="A9" s="11" t="str">
-        <x:v>Movimentos / linhas</x:v>
-      </x:c>
-      <x:c r="B9" s="8" t="str">
-        <x:v>11 movimentos / 12 linhas</x:v>
-      </x:c>
+      <x:c r="G8" s="2"/>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="2"/>
+      <x:c r="B9" s="2"/>
       <x:c r="C9" s="2"/>
-      <x:c r="D9" s="11" t="str">
-        <x:v>Conciliação</x:v>
-      </x:c>
-      <x:c r="E9" s="17" t="str">
-        <x:f>IF(ROUND(E6-E8,2)=0,"OK","DIVERGENTE")</x:f>
-        <x:v>OK</x:v>
+      <x:c r="D9" s="8" t="str">
+        <x:v>Diferença de saldo</x:v>
+      </x:c>
+      <x:c r="E9" s="11" t="n">
+        <x:f>ROUND(E7-E8,2)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F9" s="2"/>
-    </x:row>
-    <x:row r="10" ht="22" customHeight="1">
+      <x:c r="G9" s="2"/>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="2"/>
       <x:c r="B10" s="2"/>
       <x:c r="C10" s="2"/>
       <x:c r="D10" s="2"/>
       <x:c r="E10" s="2"/>
       <x:c r="F10" s="2"/>
-    </x:row>
-    <x:row r="11" ht="22" customHeight="1">
-      <x:c r="A11" s="18" t="str">
-        <x:v>ILUSTRAÇÃO PÚBLICA - NÃO UTILIZAR COMO DOCUMENTO CONTÁBIL</x:v>
-      </x:c>
-      <x:c r="B11" s="18"/>
-      <x:c r="C11" s="18"/>
-      <x:c r="D11" s="18"/>
-      <x:c r="E11" s="18"/>
-      <x:c r="F11" s="18"/>
-    </x:row>
-    <x:row r="12" ht="30" customHeight="1">
-      <x:c r="A12" s="20" t="str">
+      <x:c r="G10" s="2"/>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="15" t="str">
+        <x:v>DADOS FICTÍCIOS - NÃO UTILIZAR COMO DOCUMENTO CONTÁBIL</x:v>
+      </x:c>
+      <x:c r="B11" s="15"/>
+      <x:c r="C11" s="15"/>
+      <x:c r="D11" s="15"/>
+      <x:c r="E11" s="15"/>
+      <x:c r="F11" s="15"/>
+      <x:c r="G11" s="15"/>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="18" t="str">
         <x:v>TIPO</x:v>
       </x:c>
-      <x:c r="B12" s="20" t="str">
+      <x:c r="B12" s="18" t="str">
         <x:v>DATA</x:v>
       </x:c>
-      <x:c r="C12" s="20" t="str">
+      <x:c r="C12" s="18" t="str">
         <x:v>VALOR</x:v>
       </x:c>
-      <x:c r="D12" s="20" t="str">
+      <x:c r="D12" s="18" t="str">
         <x:v>DESCRIÇÃO</x:v>
       </x:c>
-      <x:c r="E12" s="20" t="str">
+      <x:c r="E12" s="18" t="str">
         <x:v>CATEGORIA</x:v>
       </x:c>
-      <x:c r="F12" s="20" t="str">
+      <x:c r="F12" s="18" t="str">
         <x:v>BASE DO EXEMPLO</x:v>
       </x:c>
-    </x:row>
-    <x:row r="13" ht="36" customHeight="1">
+      <x:c r="G12" s="18" t="str">
+        <x:v>DOCUMENTOS ILUSTRATIVOS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A13" s="26" t="str">
         <x:v>PAYMENT</x:v>
       </x:c>
@@ -661,31 +639,37 @@
       <x:c r="E13" s="29" t="str">
         <x:v>ADIANTAMENTO A FORNECEDORES</x:v>
       </x:c>
-      <x:c r="F13" s="28" t="n">
+      <x:c r="F13" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
-    </x:row>
-    <x:row r="14" ht="36" customHeight="1">
-      <x:c r="A14" s="34" t="str">
+      <x:c r="G13" s="29" t="str">
+        <x:v>EXEMPLO FICTÍCIO: DOC-001. Nota fiscal a receber; pendência liberada no cenário ilustrativo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="36" t="str">
         <x:v>PAYMENT</x:v>
       </x:c>
-      <x:c r="B14" s="35" t="d">
+      <x:c r="B14" s="37" t="d">
         <x:v>2026-09-04T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C14" s="36" t="n">
+      <x:c r="C14" s="38" t="n">
         <x:v>-900</x:v>
       </x:c>
-      <x:c r="D14" s="37" t="str">
+      <x:c r="D14" s="39" t="str">
         <x:v>Administrador de demonstração - pró-labore.</x:v>
       </x:c>
-      <x:c r="E14" s="37" t="str">
+      <x:c r="E14" s="39" t="str">
         <x:v>PRÓ-LABORE</x:v>
       </x:c>
-      <x:c r="F14" s="36" t="n">
+      <x:c r="F14" s="40" t="n">
         <x:v>0</x:v>
       </x:c>
-    </x:row>
-    <x:row r="15" ht="36" customHeight="1">
+      <x:c r="G14" s="39" t="str">
+        <x:v>EXEMPLO FICTÍCIO: DOC-002.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="26" t="str">
         <x:v>CREDIT</x:v>
       </x:c>
@@ -701,31 +685,37 @@
       <x:c r="E15" s="29" t="str">
         <x:v>RECEITA ALUGUÉIS</x:v>
       </x:c>
-      <x:c r="F15" s="28" t="n">
+      <x:c r="F15" s="30" t="n">
         <x:v>2300</x:v>
       </x:c>
-    </x:row>
-    <x:row r="16" ht="36" customHeight="1">
-      <x:c r="A16" s="34" t="str">
+      <x:c r="G15" s="29" t="str">
+        <x:v>EXEMPLO FICTÍCIO: DOC-003.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="36" t="str">
         <x:v>PAYMENT</x:v>
       </x:c>
-      <x:c r="B16" s="35" t="d">
+      <x:c r="B16" s="37" t="d">
         <x:v>2026-09-08T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C16" s="36" t="n">
+      <x:c r="C16" s="38" t="n">
         <x:v>-120</x:v>
       </x:c>
-      <x:c r="D16" s="37" t="str">
+      <x:c r="D16" s="39" t="str">
         <x:v>PIS - parcela de pagamento conjunto fictício de R$ 620,00.</x:v>
       </x:c>
-      <x:c r="E16" s="37" t="str">
+      <x:c r="E16" s="39" t="str">
         <x:v>IMPOSTOS FEDERAIS - PIS</x:v>
       </x:c>
-      <x:c r="F16" s="36" t="n">
+      <x:c r="F16" s="40" t="n">
         <x:v>0</x:v>
       </x:c>
-    </x:row>
-    <x:row r="17" ht="36" customHeight="1">
+      <x:c r="G16" s="39" t="str">
+        <x:v>EXEMPLO FICTÍCIO: DOC-004. Mesmo movimento da parcela COFINS.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="26" t="str">
         <x:v>PAYMENT</x:v>
       </x:c>
@@ -741,31 +731,37 @@
       <x:c r="E17" s="29" t="str">
         <x:v>IMPOSTOS FEDERAIS - COFINS</x:v>
       </x:c>
-      <x:c r="F17" s="28" t="n">
+      <x:c r="F17" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
-    </x:row>
-    <x:row r="18" ht="36" customHeight="1">
-      <x:c r="A18" s="34" t="str">
+      <x:c r="G17" s="29" t="str">
+        <x:v>EXEMPLO FICTÍCIO: DOC-004. PIS + COFINS = R$ 620,00.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="36" t="str">
         <x:v>CREDIT</x:v>
       </x:c>
-      <x:c r="B18" s="35" t="d">
+      <x:c r="B18" s="37" t="d">
         <x:v>2026-09-10T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C18" s="36" t="n">
+      <x:c r="C18" s="38" t="n">
         <x:v>3400</x:v>
       </x:c>
-      <x:c r="D18" s="37" t="str">
+      <x:c r="D18" s="39" t="str">
         <x:v>Locatário Beta - aluguel do período.</x:v>
       </x:c>
-      <x:c r="E18" s="37" t="str">
+      <x:c r="E18" s="39" t="str">
         <x:v>RECEITA ALUGUÉIS</x:v>
       </x:c>
-      <x:c r="F18" s="36" t="n">
+      <x:c r="F18" s="40" t="n">
         <x:v>3400</x:v>
       </x:c>
-    </x:row>
-    <x:row r="19" ht="36" customHeight="1">
+      <x:c r="G18" s="39" t="str">
+        <x:v>EXEMPLO FICTÍCIO: DOC-005.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="26" t="str">
         <x:v>PAYMENT</x:v>
       </x:c>
@@ -781,31 +777,37 @@
       <x:c r="E19" s="29" t="str">
         <x:v>PLANO DE SAÚDE</x:v>
       </x:c>
-      <x:c r="F19" s="28" t="n">
+      <x:c r="F19" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
-    </x:row>
-    <x:row r="20" ht="36" customHeight="1">
-      <x:c r="A20" s="34" t="str">
+      <x:c r="G19" s="29" t="str">
+        <x:v>EXEMPLO FICTÍCIO: DOC-006.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A20" s="36" t="str">
         <x:v>CREDIT</x:v>
       </x:c>
-      <x:c r="B20" s="35" t="d">
+      <x:c r="B20" s="37" t="d">
         <x:v>2026-09-15T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C20" s="36" t="n">
+      <x:c r="C20" s="38" t="n">
         <x:v>7500</x:v>
       </x:c>
-      <x:c r="D20" s="37" t="str">
+      <x:c r="D20" s="39" t="str">
         <x:v>Seguradora Exemplo - ressarcimento para reparo.</x:v>
       </x:c>
-      <x:c r="E20" s="37" t="str">
+      <x:c r="E20" s="39" t="str">
         <x:v>RESSARCIMENTO/INDENIZAÇÃO DE SEGURO</x:v>
       </x:c>
-      <x:c r="F20" s="36" t="n">
+      <x:c r="F20" s="40" t="n">
         <x:v>0</x:v>
       </x:c>
-    </x:row>
-    <x:row r="21" ht="36" customHeight="1">
+      <x:c r="G20" s="39" t="str">
+        <x:v>EXEMPLO FICTÍCIO: DOC-007. Fora da base apenas no cenário demonstrado.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="26" t="str">
         <x:v>PAYMENT</x:v>
       </x:c>
@@ -821,31 +823,37 @@
       <x:c r="E21" s="29" t="str">
         <x:v>CONTABILIDADE</x:v>
       </x:c>
-      <x:c r="F21" s="28" t="n">
+      <x:c r="F21" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
-    </x:row>
-    <x:row r="22" ht="36" customHeight="1">
-      <x:c r="A22" s="34" t="str">
+      <x:c r="G21" s="29" t="str">
+        <x:v>EXEMPLO FICTÍCIO: DOC-008.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="36" t="str">
         <x:v>PAYMENT</x:v>
       </x:c>
-      <x:c r="B22" s="35" t="d">
+      <x:c r="B22" s="37" t="d">
         <x:v>2026-09-20T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C22" s="36" t="n">
+      <x:c r="C22" s="38" t="n">
         <x:v>-1000</x:v>
       </x:c>
-      <x:c r="D22" s="37" t="str">
+      <x:c r="D22" s="39" t="str">
         <x:v>Aplicação financeira de demonstração.</x:v>
       </x:c>
-      <x:c r="E22" s="37" t="str">
+      <x:c r="E22" s="39" t="str">
         <x:v>APLICAÇÕES FINANCEIRAS</x:v>
       </x:c>
-      <x:c r="F22" s="36" t="n">
+      <x:c r="F22" s="40" t="n">
         <x:v>0</x:v>
       </x:c>
-    </x:row>
-    <x:row r="23" ht="36" customHeight="1">
+      <x:c r="G22" s="39" t="str">
+        <x:v>EXEMPLO FICTÍCIO: DOC-009.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="26" t="str">
         <x:v>PAYMENT</x:v>
       </x:c>
@@ -861,122 +869,157 @@
       <x:c r="E23" s="29" t="str">
         <x:v>DISTRIBUIÇÃO DE LUCROS</x:v>
       </x:c>
-      <x:c r="F23" s="28" t="n">
+      <x:c r="F23" s="30" t="n">
         <x:v>0</x:v>
       </x:c>
-    </x:row>
-    <x:row r="24" ht="36" customHeight="1">
-      <x:c r="A24" s="34" t="str">
+      <x:c r="G23" s="29" t="str">
+        <x:v>EXEMPLO FICTÍCIO: DOC-010.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
+      <x:c r="A24" s="36" t="str">
         <x:v>CREDIT</x:v>
       </x:c>
-      <x:c r="B24" s="35" t="d">
+      <x:c r="B24" s="37" t="d">
         <x:v>2026-09-28T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C24" s="36" t="n">
+      <x:c r="C24" s="38" t="n">
         <x:v>1800</x:v>
       </x:c>
-      <x:c r="D24" s="37" t="str">
+      <x:c r="D24" s="39" t="str">
         <x:v>Locatário Gama - aluguel do período.</x:v>
       </x:c>
-      <x:c r="E24" s="37" t="str">
+      <x:c r="E24" s="39" t="str">
         <x:v>RECEITA ALUGUÉIS</x:v>
       </x:c>
-      <x:c r="F24" s="36" t="n">
+      <x:c r="F24" s="40" t="n">
         <x:v>1800</x:v>
       </x:c>
-    </x:row>
-    <x:row r="25" ht="28" customHeight="1">
+      <x:c r="G24" s="39" t="str">
+        <x:v>EXEMPLO FICTÍCIO: DOC-011.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="15" hidden="0" customHeight="1">
       <x:c r="A25" s="2"/>
       <x:c r="B25" s="2"/>
       <x:c r="C25" s="2"/>
       <x:c r="D25" s="2"/>
-      <x:c r="E25" s="39" t="str">
+      <x:c r="E25" s="6" t="str">
         <x:v>TOTAL DA BASE DO EXEMPLO</x:v>
       </x:c>
-      <x:c r="F25" s="40" t="n">
+      <x:c r="F25" s="13" t="n">
         <x:f>ROUND(SUM(F13:F24),2)</x:f>
         <x:v>7500</x:v>
       </x:c>
-    </x:row>
-    <x:row r="26" ht="22" customHeight="1">
+      <x:c r="G25" s="2"/>
+    </x:row>
+    <x:row r="26" ht="15" hidden="0" customHeight="1">
       <x:c r="A26" s="2"/>
       <x:c r="B26" s="2"/>
       <x:c r="C26" s="2"/>
       <x:c r="D26" s="2"/>
       <x:c r="E26" s="2"/>
       <x:c r="F26" s="2"/>
-    </x:row>
-    <x:row r="27" ht="26" customHeight="1">
-      <x:c r="A27" s="42" t="str">
-        <x:v>11 movimentos bancários em 12 linhas: o pagamento de R$ 620,00 foi separado em PIS (R$ 120,00) e COFINS (R$ 500,00), sem duplicar valores.</x:v>
-      </x:c>
-      <x:c r="B27" s="42"/>
-      <x:c r="C27" s="42"/>
-      <x:c r="D27" s="42"/>
-      <x:c r="E27" s="42"/>
-      <x:c r="F27" s="42"/>
-    </x:row>
-    <x:row r="28" ht="26" customHeight="1">
-      <x:c r="A28" s="42" t="str">
-        <x:v>A base de R$ 7.500,00 inclui apenas os três aluguéis neste cenário fictício. O ressarcimento fica fora da base exclusivamente nesta ilustração.</x:v>
-      </x:c>
-      <x:c r="B28" s="42"/>
-      <x:c r="C28" s="42"/>
-      <x:c r="D28" s="42"/>
-      <x:c r="E28" s="42"/>
-      <x:c r="F28" s="42"/>
-    </x:row>
-    <x:row r="29" ht="26" customHeight="1">
-      <x:c r="A29" s="42" t="str">
-        <x:v>O adiantamento ao Fornecedor Modelo tem nota fiscal pendente neste cenário. Não há documentos reais associados aos lançamentos.</x:v>
-      </x:c>
-      <x:c r="B29" s="42"/>
-      <x:c r="C29" s="42"/>
-      <x:c r="D29" s="42"/>
-      <x:c r="E29" s="42"/>
-      <x:c r="F29" s="42"/>
-    </x:row>
-    <x:row r="30" ht="26" customHeight="1">
-      <x:c r="A30" s="42" t="str">
-        <x:v>Exemplo construído com dados sintéticos para ilustrar a entrega; não representa nova execução sobre comprovantes públicos nem orientação fiscal.</x:v>
-      </x:c>
-      <x:c r="B30" s="42"/>
-      <x:c r="C30" s="42"/>
-      <x:c r="D30" s="42"/>
-      <x:c r="E30" s="42"/>
-      <x:c r="F30" s="42"/>
-    </x:row>
-    <x:row r="31" ht="26" customHeight="1">
-      <x:c r="A31" s="42" t="str">
-        <x:v>SmartChat na prática: https://github.com/ubirajaratheodoro/smartchat/tree/main/na-pratica/conciliacao-financeira</x:v>
-      </x:c>
-      <x:c r="B31" s="42"/>
-      <x:c r="C31" s="42"/>
-      <x:c r="D31" s="42"/>
-      <x:c r="E31" s="42"/>
-      <x:c r="F31" s="42"/>
-    </x:row>
-    <x:row r="32" ht="26" customHeight="1">
-      <x:c r="A32" s="42" t="str">
-        <x:v>Padrão de especificação (link provisório): https://sun.eduzz.com/Q9NDKAYP01</x:v>
-      </x:c>
-      <x:c r="B32" s="42"/>
-      <x:c r="C32" s="42"/>
-      <x:c r="D32" s="42"/>
-      <x:c r="E32" s="42"/>
-      <x:c r="F32" s="42"/>
+      <x:c r="G26" s="2"/>
+    </x:row>
+    <x:row r="27" ht="15" hidden="0" customHeight="1">
+      <x:c r="A27" s="10" t="str">
+        <x:v>COMO LER ESTE EXEMPLO</x:v>
+      </x:c>
+      <x:c r="B27" s="10"/>
+      <x:c r="C27" s="10"/>
+      <x:c r="D27" s="10"/>
+      <x:c r="E27" s="10"/>
+      <x:c r="F27" s="10"/>
+      <x:c r="G27" s="10"/>
+    </x:row>
+    <x:row r="28" ht="15" hidden="0" customHeight="1">
+      <x:c r="A28" s="6" t="str">
+        <x:v>Esta planilha foi construída exclusivamente com dados sintéticos para ilustrar uma entrega. Não é o resultado de uma nova execução sobre comprovantes públicos.</x:v>
+      </x:c>
+      <x:c r="B28" s="6"/>
+      <x:c r="C28" s="6"/>
+      <x:c r="D28" s="6"/>
+      <x:c r="E28" s="6"/>
+      <x:c r="F28" s="6"/>
+      <x:c r="G28" s="6"/>
+    </x:row>
+    <x:row r="29" ht="15" hidden="0" customHeight="1">
+      <x:c r="A29" s="6" t="str">
+        <x:v>Um movimento de pagamento de R$ 620,00 é mostrado em duas linhas: PIS de R$ 120,00 e COFINS de R$ 500,00. Assim, 11 movimentos aparecem em 12 linhas, sem dupla contagem.</x:v>
+      </x:c>
+      <x:c r="B29" s="6"/>
+      <x:c r="C29" s="6"/>
+      <x:c r="D29" s="6"/>
+      <x:c r="E29" s="6"/>
+      <x:c r="F29" s="6"/>
+      <x:c r="G29" s="6"/>
+    </x:row>
+    <x:row r="30" ht="15" hidden="0" customHeight="1">
+      <x:c r="A30" s="6" t="str">
+        <x:v>A base de R$ 7.500,00 inclui apenas os três aluguéis neste cenário inventado. A exclusão do ressarcimento não estabelece orientação tributária para casos reais.</x:v>
+      </x:c>
+      <x:c r="B30" s="6"/>
+      <x:c r="C30" s="6"/>
+      <x:c r="D30" s="6"/>
+      <x:c r="E30" s="6"/>
+      <x:c r="F30" s="6"/>
+      <x:c r="G30" s="6"/>
+    </x:row>
+    <x:row r="31" ht="15" hidden="0" customHeight="1">
+      <x:c r="A31" s="6" t="str">
+        <x:v>Os identificadores DOC-001 a DOC-011 são fictícios. Não existem arquivos, contas, pessoas ou links reais associados a eles.</x:v>
+      </x:c>
+      <x:c r="B31" s="6"/>
+      <x:c r="C31" s="6"/>
+      <x:c r="D31" s="6"/>
+      <x:c r="E31" s="6"/>
+      <x:c r="F31" s="6"/>
+      <x:c r="G31" s="6"/>
+    </x:row>
+    <x:row r="32" ht="15" hidden="0" customHeight="1">
+      <x:c r="A32" s="6" t="str">
+        <x:v>Conheça a aplicação e o SmartChat: https://github.com/ubirajaratheodoro/smartchat/tree/main/na-pratica/conciliacao-financeira</x:v>
+      </x:c>
+      <x:c r="B32" s="6"/>
+      <x:c r="C32" s="6"/>
+      <x:c r="D32" s="6"/>
+      <x:c r="E32" s="6"/>
+      <x:c r="F32" s="6"/>
+      <x:c r="G32" s="6"/>
+    </x:row>
+    <x:row r="33" ht="15" hidden="0" customHeight="1">
+      <x:c r="A33" s="6" t="str">
+        <x:v>Padrão de especificação: https://sun.eduzz.com/Q9NDKAYP01</x:v>
+      </x:c>
+      <x:c r="B33" s="6"/>
+      <x:c r="C33" s="6"/>
+      <x:c r="D33" s="6"/>
+      <x:c r="E33" s="6"/>
+      <x:c r="F33" s="6"/>
+      <x:c r="G33" s="6"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="2"/>
+      <x:c r="B34" s="2"/>
+      <x:c r="C34" s="2"/>
+      <x:c r="D34" s="2"/>
+      <x:c r="E34" s="2"/>
+      <x:c r="F34" s="2"/>
+      <x:c r="G34" s="2"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:F1"/>
-    <x:mergeCell ref="A2:F2"/>
-    <x:mergeCell ref="A11:F11"/>
-    <x:mergeCell ref="A27:F27"/>
-    <x:mergeCell ref="A28:F28"/>
-    <x:mergeCell ref="A29:F29"/>
-    <x:mergeCell ref="A30:F30"/>
-    <x:mergeCell ref="A31:F31"/>
-    <x:mergeCell ref="A32:F32"/>
+    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A2:G2"/>
+    <x:mergeCell ref="A11:G11"/>
+    <x:mergeCell ref="A27:G27"/>
+    <x:mergeCell ref="A28:G28"/>
+    <x:mergeCell ref="A29:G29"/>
+    <x:mergeCell ref="A30:G30"/>
+    <x:mergeCell ref="A31:G31"/>
+    <x:mergeCell ref="A32:G32"/>
+    <x:mergeCell ref="A33:G33"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>